<commit_message>
H2 storage + uncertainty in demand
</commit_message>
<xml_diff>
--- a/data/processed/params.xlsx
+++ b/data/processed/params.xlsx
@@ -1,31 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Miriam Ucendo\Documents\UNI\5\TFG_mates\code\EH2_mod\nuevo\data\processed\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Miriam Ucendo\Documents\UNI\5\practicas\OEH\1605136_BSc_Math\data\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60A1480D-9BC5-40A6-9750-39FF2E70F2D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56E316DB-BCE4-42F4-9156-A6426FEA35E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>Name</t>
   </si>
@@ -97,6 +108,27 @@
   </si>
   <si>
     <t>H_EHP_max</t>
+  </si>
+  <si>
+    <t>eta_F</t>
+  </si>
+  <si>
+    <t>el_max</t>
+  </si>
+  <si>
+    <t>fc_max</t>
+  </si>
+  <si>
+    <t>SOC_H2_ini</t>
+  </si>
+  <si>
+    <t>SOC_H2_min</t>
+  </si>
+  <si>
+    <t>SOC_H2_max</t>
+  </si>
+  <si>
+    <t>eta_EL</t>
   </si>
 </sst>
 </file>
@@ -452,10 +484,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -642,6 +674,64 @@
         <v>500</v>
       </c>
     </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26">
+        <f>0.8*500</f>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27">
+        <f>0.1*500</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>500</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add stochastic model EH5, visual diagram, and run files
</commit_message>
<xml_diff>
--- a/data/processed/params.xlsx
+++ b/data/processed/params.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Miriam Ucendo\Documents\UNI\5\practicas\OEH\1605136_BSc_Math\data\processed\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Miriam Ucendo\Documents\UNI\5\practicas\OEH\OEH_SO\data\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56E316DB-BCE4-42F4-9156-A6426FEA35E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28CDA2D7-741B-4E53-A6C0-9DA0164EF5AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
   <si>
     <t>Name</t>
   </si>
@@ -129,6 +129,90 @@
   </si>
   <si>
     <t>eta_EL</t>
+  </si>
+  <si>
+    <t>p_stb</t>
+  </si>
+  <si>
+    <t>h_warmup</t>
+  </si>
+  <si>
+    <t>el_min</t>
+  </si>
+  <si>
+    <t>fc_min</t>
+  </si>
+  <si>
+    <t>eta_H2</t>
+  </si>
+  <si>
+    <t>alpha_DES</t>
+  </si>
+  <si>
+    <t>(furnace)</t>
+  </si>
+  <si>
+    <t>(CHP)</t>
+  </si>
+  <si>
+    <t>ramp_up_el</t>
+  </si>
+  <si>
+    <t>ramp_down_el</t>
+  </si>
+  <si>
+    <t>( 45% el_max / h, Hassan et al. 2026 )</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ( 45% el_max / h, Hassan et al. 2026 )</t>
+  </si>
+  <si>
+    <t>( 30% el_max, Liao et al. 2026 / SOEC )</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ( nominal capacity )</t>
+  </si>
+  <si>
+    <t>( 5.5% el_max, Liao et al. 2026 )</t>
+  </si>
+  <si>
+    <t>eta_com</t>
+  </si>
+  <si>
+    <t>rho_com</t>
+  </si>
+  <si>
+    <t>ramp_down_F</t>
+  </si>
+  <si>
+    <t>ramp_up_F</t>
+  </si>
+  <si>
+    <t>(capacity )</t>
+  </si>
+  <si>
+    <t>( 0.07% el_max, Shi et al. 2025 )</t>
+  </si>
+  <si>
+    <t>( 2.2 kWh/kg at 200 bar, Tian et al. 2024 / Shi et al. 2025 )</t>
+  </si>
+  <si>
+    <t>( 85% compressor efficiency, Tian et al. 2023 / Shi et al. 2025 )</t>
+  </si>
+  <si>
+    <t>( 70% fuel cell efficiency, Hassan et al. 2026 / Shi et al. 2025 )</t>
+  </si>
+  <si>
+    <t>( 10% fc_max, Shi et al. 2025 / Hassan et al. 2026 )</t>
+  </si>
+  <si>
+    <t>( nominal fuel cell capacity, 50% el_max )</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ( 100% fc_max / h, Hassan et al. 2026 )</t>
+  </si>
+  <si>
+    <t>( 100% fc_max / h, Hassan et al. 2026 )</t>
   </si>
 </sst>
 </file>
@@ -162,7 +246,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -172,6 +256,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -193,12 +289,16 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Millares 2" xfId="4" xr:uid="{579E00ED-6BE0-4FD7-9C1F-1A0D60A42D05}"/>
@@ -484,13 +584,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -498,241 +598,395 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>0.35</v>
+      </c>
+      <c r="C4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5">
+        <v>0.9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="2">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="2">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B13" s="2">
         <v>1000</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B14" s="2">
         <v>120</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B15" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="4">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17">
+        <f>0.3*B18</f>
+        <v>30</v>
+      </c>
+      <c r="C17" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" s="7">
+        <v>100</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>31</v>
+      </c>
+      <c r="B19">
+        <f>0.055*B18</f>
+        <v>5.5</v>
+      </c>
+      <c r="C19" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20">
+        <f>0.45*B18</f>
+        <v>45</v>
+      </c>
+      <c r="C20" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21">
+        <f>0.45*B18</f>
+        <v>45</v>
+      </c>
+      <c r="C21" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>32</v>
+      </c>
+      <c r="B22">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B23">
+        <f>0.0007*B18</f>
+        <v>6.9999999999999993E-2</v>
+      </c>
+      <c r="C23" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24">
+        <v>0.85</v>
+      </c>
+      <c r="C24" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B25">
+        <v>2.2000000000000001E-3</v>
+      </c>
+      <c r="C25" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26">
+        <v>0.7</v>
+      </c>
+      <c r="C26" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27">
+        <f>0.1*B28</f>
         <v>5</v>
       </c>
-      <c r="B5">
-        <v>0.99</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>0.99</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7">
+      <c r="C27" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28">
+        <f>0.5*B18</f>
+        <v>50</v>
+      </c>
+      <c r="C28" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B29">
+        <f>B28</f>
+        <v>50</v>
+      </c>
+      <c r="C29" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B30">
+        <f>B28</f>
+        <v>50</v>
+      </c>
+      <c r="C30" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B31">
         <v>0.98</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8">
-        <v>0.45</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
-        <v>0.35</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10">
-        <v>0.95</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B32">
+        <f>0.01*B33</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B33">
+        <v>500</v>
+      </c>
+      <c r="C33" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B34">
+        <f>0.01*B33</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B35" s="2">
         <v>250</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B36" s="2">
         <v>500</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B37" s="2">
         <v>600</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>15</v>
-      </c>
-      <c r="B15" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>16</v>
-      </c>
-      <c r="B16" s="2">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>17</v>
-      </c>
-      <c r="B17" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18" s="2">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="3">
+      <c r="B38" s="3">
         <v>2.5</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="4">
+      <c r="B39" s="4">
         <v>0.01</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B40" s="2">
         <v>500</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B22">
+      <c r="B41">
         <v>0.01</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B23">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>30</v>
-      </c>
-      <c r="B24">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>24</v>
-      </c>
-      <c r="B25">
-        <v>0.7</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>25</v>
-      </c>
-      <c r="B26">
-        <f>0.8*500</f>
-        <v>400</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>26</v>
-      </c>
-      <c r="B27">
-        <f>0.1*500</f>
-        <v>50</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>27</v>
-      </c>
-      <c r="B28">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>28</v>
-      </c>
-      <c r="B29">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>29</v>
-      </c>
-      <c r="B30">
+      <c r="B42">
         <v>500</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>